<commit_message>
Implement create Aktuelle_angebote sheet & import Angebotsformular & create Ablieferungsverzeichnis & replace and rename documents in Vorlage
</commit_message>
<xml_diff>
--- a/Daten/Stammdaten.xlsx
+++ b/Daten/Stammdaten.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\08_Zwischenablage_Mitarbeiter\Changten_Tseten_cen\Projekte\Ablieferungsmakro\Daten\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\home.kt.ktzh.ch\BAA7556$\Desktop\Projects\delivery-macro\Daten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE201F9B-C52A-4C88-A933-05D4CCAF0802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD74071-D3B0-4DF7-9873-CCCD7C6D517E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A81106D9-307E-4571-99B3-1C4A9B6F97E7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A81106D9-307E-4571-99B3-1C4A9B6F97E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Dateipfade" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="70">
   <si>
     <t>Pfad zu Ablieferungsvereinbarung-Vorlage:</t>
   </si>
@@ -238,19 +238,16 @@
     <t>Pfad zu Angebotstabelle-Vorlage:</t>
   </si>
   <si>
-    <t>\Vorlagen\Ablieferungsverzeichnis, Vorlage.dotx</t>
-  </si>
-  <si>
-    <t>\Vorlagen\Aktenangebotsformular, Vorlage.docx</t>
-  </si>
-  <si>
-    <t>\Vorlagen\Ablieferungsverzeichnis, Vorlage.xltx</t>
-  </si>
-  <si>
-    <t>\Vorlagen\Ablieferungsvereinbarung, Vorlage.dotx</t>
-  </si>
-  <si>
-    <t>\Vorlagen\Angebotstabelle, Vorlage.xlsx</t>
+    <t>./Vorlagen/Aktenangebotsformular, Vorlage.docx</t>
+  </si>
+  <si>
+    <t>./Vorlagen/Angebotstabelle, Vorlage.xlsx</t>
+  </si>
+  <si>
+    <t>./Vorlagen/Ablieferungsvereinbarung, Vorlage.docx</t>
+  </si>
+  <si>
+    <t>./Vorlagen/Ablieferungsverzeichnis, Vorlage.xlsx</t>
   </si>
 </sst>
 </file>
@@ -835,7 +832,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{963B26AF-C922-41E9-B9CC-ECF59C79EDFC}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -847,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.25">
@@ -855,7 +852,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.25">
@@ -863,23 +860,15 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement create deliveryList & fix errors of date & add in deliveryAgreement contact and new line after year
</commit_message>
<xml_diff>
--- a/Daten/Stammdaten.xlsx
+++ b/Daten/Stammdaten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\home.kt.ktzh.ch\BAA7556$\Desktop\Projects\delivery-macro\Daten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD74071-D3B0-4DF7-9873-CCCD7C6D517E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F52C6C-803F-4B80-8D69-3B13D5FEC4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A81106D9-307E-4571-99B3-1C4A9B6F97E7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A81106D9-307E-4571-99B3-1C4A9B6F97E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Dateipfade" sheetId="1" r:id="rId1"/>
@@ -241,13 +241,13 @@
     <t>./Vorlagen/Aktenangebotsformular, Vorlage.docx</t>
   </si>
   <si>
+    <t>./Vorlagen/Ablieferungsvereinbarung, Vorlage.docx</t>
+  </si>
+  <si>
+    <t>./Vorlagen/Ablieferungsverzeichnis, Vorlage.xlsx</t>
+  </si>
+  <si>
     <t>./Vorlagen/Angebotstabelle, Vorlage.xlsx</t>
-  </si>
-  <si>
-    <t>./Vorlagen/Ablieferungsvereinbarung, Vorlage.docx</t>
-  </si>
-  <si>
-    <t>./Vorlagen/Ablieferungsverzeichnis, Vorlage.xlsx</t>
   </si>
 </sst>
 </file>
@@ -844,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.25">
@@ -852,7 +852,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.25">
@@ -868,7 +868,7 @@
         <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add complete config file & fix/edit services & remove mark code and write logic in excel file
</commit_message>
<xml_diff>
--- a/Daten/Stammdaten.xlsx
+++ b/Daten/Stammdaten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\home.kt.ktzh.ch\BAA7556$\Desktop\Projects\delivery-macro\Daten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F52C6C-803F-4B80-8D69-3B13D5FEC4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B17F5E-7361-433F-9CE8-F57DB192C356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A81106D9-307E-4571-99B3-1C4A9B6F97E7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A81106D9-307E-4571-99B3-1C4A9B6F97E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Dateipfade" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Create readme & change folderstructure & delete libs because venv is working & change vba call for scripts
</commit_message>
<xml_diff>
--- a/Daten/Stammdaten.xlsx
+++ b/Daten/Stammdaten.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\home.kt.ktzh.ch\BAA7556$\Desktop\Projects\delivery-macro\Daten\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B17F5E-7361-433F-9CE8-F57DB192C356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54DFDBB7-84D5-42BD-ADF6-ECD8E74D85EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A81106D9-307E-4571-99B3-1C4A9B6F97E7}"/>
   </bookViews>
@@ -238,13 +238,13 @@
     <t>Pfad zu Angebotstabelle-Vorlage:</t>
   </si>
   <si>
+    <t>./Vorlagen/Ablieferungsvereinbarung, Vorlage.docx</t>
+  </si>
+  <si>
+    <t>./Vorlagen/Ablieferungsverzeichnis, Vorlage.xlsx</t>
+  </si>
+  <si>
     <t>./Vorlagen/Aktenangebotsformular, Vorlage.docx</t>
-  </si>
-  <si>
-    <t>./Vorlagen/Ablieferungsvereinbarung, Vorlage.docx</t>
-  </si>
-  <si>
-    <t>./Vorlagen/Ablieferungsverzeichnis, Vorlage.xlsx</t>
   </si>
   <si>
     <t>./Vorlagen/Angebotstabelle, Vorlage.xlsx</t>
@@ -844,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.25">
@@ -852,7 +852,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.25">
@@ -860,7 +860,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.25">

</xml_diff>